<commit_message>
Inventario al 20.10.2026 y acceso por correo autorizado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ASsM9mcqYrhrTsJC3CpHT
</commit_message>
<xml_diff>
--- a/plantillas/103.xlsx
+++ b/plantillas/103.xlsx
@@ -12096,7 +12096,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -12536,7 +12536,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -12656,7 +12656,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -13074,7 +13074,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>19.10.2026</t>
+          <t>20.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>